<commit_message>
fix: weekly report classify_news adapts to dict-format tags
</commit_message>
<xml_diff>
--- a/weekly_temp/patents_量子软件与算法.xlsx
+++ b/weekly_temp/patents_量子软件与算法.xlsx
@@ -456,17 +456,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>量子计算控制装置、量子计算机及量子计算控制方法</t>
+          <t>学习装置、数据处理装置、参数生成装置、学习方法、数据处理方法和参数生成方法</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>独立行政法人科学技术振兴机构</t>
+          <t>索尼集团公司</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>中村泰信 | 田渊丰 | 玉手修平</t>
+          <t>INAISHI, DAISUKE | ARAI, HIROAKI | HIRAI, YUMA | KOSAKA, JUNICHI | KANAO, RINNA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,184 +476,182 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>量子计算控制装置具备控制信号生成部和量子比特模块。量子比特模块具备观测部、量子比特基板部、控制电路部、观测电路部以及信号处理电路部。多个量子比特分组为由各量子比特彼此的位置关系相同的多个量子比特构成的多个组而配置在量子比特基板部上。控制信号生成部生成控制信号和命令信号，控制信号用于执行一个以上的种类的空间上均匀的第一操作及以比一个以上的种类的第一操作低的频度来进行的空间上不均匀的第二操作，命令信号用于使控制电路部执行第一操作及第二操作的控制，该第一操作及第二操作是针对量子比特基板部上的量子比特的操作。控制电路部将控制信号分支到组，根据命令信号，对控制信号向量子比特基板部上的各量子比特的送出进行控制。观测电路部观测接受了第一操作或第二操作的各量子比特的状态。信号处理电路部向观测部发送各量子比特的观测信号。</t>
+          <t>在学习装置(10)中,第一评估单元(14)对多个图像数据进行定量评估,从而获取针对多个图像数据中的每一个的多个第一评估结果;教师数据生成单元(15)基于多个第一评估结果,从具有彼此不同值的多个第一参数中选择第二参数,并生成包括所选第二参数的第一组教师数据;第一机器学习单元(17)使用第一组教师数据进行机器学习,从而生成输出用于处理处理目标的图像数据的第三参数的学习模型。</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=efec951d-1740-473f-842d-97180ce3a76d&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=cWStYX30VcRxj2P%2BjMY8Zcter538VTu%2BbtjG7vto470%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=09b602ca-7cd6-46b9-89a4-4e1187e8767c&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=Cngt8rv7tt158dYJYry8%2BZbNvBX8N1TGHCAHUIPW%2Fyw%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>原子的电子态分离器、原子干涉仪、原子跃迁频率测量装置、原子振荡器、光晶格钟、量子计算机及原子的电子态叠加态的生成方法</t>
+          <t>量子计算系统中的参量放大</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>国立大学法人东京大学</t>
+          <t>RIGETTI &amp; CO INC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>香取秀俊</t>
+          <t>SELVANAYAGAM,, MICHAEL KARUNENDRA | RAMACHANDRAN,, GANESH | MOHAN,, YUVRAJ | SHARAC,, NICHOLAS WARREN | FENG,, DENNIS CHEN | VAHIDPOUR,, MEHRNOOSH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>本发明的原子的电子态分离器(1)包括：原子供给部(11)、原子移动路径(12)、探测激光光源(13)和磁场生成部(M)。原子供给部(11)供给以一定速度在原子移动路径(12)中移动的原子。探测激光光源(13)向原子移动路径(12)内供给与原子移动路径(12)同轴地在与原子的运动方向相反或相同的方向上传播的探测激光。磁场生成部(M)通过在原子移动路径(12)中生成与原子移动路径(12)正交的磁场并进行与容许电偶极子跃迁的电子态的波函数混合，能够进行基于在时间和空间上同样的探测激光的时钟跃迁的脉冲激发。或者，磁屏蔽件通过屏蔽在原子移动路径(12)中施加的磁场并在空间上改变塞曼频移，从而能够通过在时间和空间上同样的探测激光对时钟跃迁进行脉冲激发。其结果，能够连续地进行原子跃迁的分光和探测激光的频率控制，提高原子钟的稳定度。</t>
+          <t>一般来说,参量放大是在量子计算系统中实现的。在某些情况下,行波参量放大器(TWPA)包含多个串联的约瑟夫森结。这些约瑟夫森结包括一个第一约瑟夫森结,该第一约瑟夫森结包括位于衬底表面上的第一超导电极、与第一超导电极重叠的第二超导电极,以及夹在第一和第二超导电极重叠部分之间的势垒。该势垒在衬底表面上形成一个锥形区域。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=826fc8c9-43e7-46de-ba8a-7944a1978dc4&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=LlykcgPkjh3vLSNIh6JaxjqICxUxQMbBk6mblb38Uwg%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=5a6b90a4-a56f-4568-9561-e3f877eac10f&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=oDm5LSn6jC86Ao1xLgF%2BCW%2BmwUGg0v9UbX26H7BQkTI%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>基于FPGA的蒙特卡罗路径积分-模拟量子退火方法及系统</t>
+          <t>利用人工智能解决特定领域问题</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>西安电子科技大学</t>
+          <t>人工天才公司</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>朱畅华 | 李帅威 | 何先灯 | 魏建涛 | 权东晓 | 易运晖 | 赵楠 | 陈南</t>
+          <t>BURCHARD, PAUL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>本发明公开了一种基于FPGA实现的蒙特卡罗路径积分‑模拟量子退火方法，主要解决现有蒙特卡罗路径积分‑模拟量子退火算法在CPU上运行时间效率低的问题，其实现方案包括:在Bram空间初始化原始矩阵；FPGA产生随机数以对原始矩阵进行随机操作得到新矩阵；并行计算新矩阵和原始矩阵势能项差值、动能项差值和哈密顿量差值；判断是否更新原始矩阵；选择执行更新操作后原始矩阵中势能项最小的矩阵作为当前的最优方案解；更新耦合系数不断进行迭代直到设定的迭代次数，得到最优解即为最终的最优路径。本发明大幅提升了运行的时间效率，相对于传统的蒙特卡罗路径积分‑模拟量子退火算法运行时间提高了79倍，可用于实时性要求高场景的无人机路由规划。</t>
+          <t>本文描述了利用人工智能为特定领域问题提供可解释解决方案的新方法。计算单元识别特定领域问题,例如生物学问题。计算单元确定一个初始特征子集,该子集包含该问题可观察特征的各种特征。计算单元优化初始特征子集,以提高该子集生成问题解决方案的准确性。计算单元基于优化后的子集训练一个或多个预测人工智能模型,以输出该问题的解决方案。随后,计算单元利用训练后的预测模型输出一个或多个其他特定领域问题的解决方案。计算单元还可以通过输出预测模型执行的步骤的表示来为特定领域的问题提供可解释的解决方案。</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=4995bc0f-40ae-45ff-a154-7460d307f8a1&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=mw%2F8XzKpXOlI5GwRkITNxI8qXk7gfaPvM1rU8BWWW%2BY%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=ed3db125-1edd-46c4-8bec-b6f6711e683e&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=%2Bp73R2mjhqlXvbjBOiG8LTALKPBFpupReNchfjFm2Rc%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>用于量子计算测控的集成滤波放大装置</t>
+          <t>利用量子纠缠的大型语言模型</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>相干(北京)科技有限公司</t>
+          <t>万事达卡国际股份有限公司</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>赵剑琴 | 邢磊 | 田建强 | 贺玉龙 | 曾祥洪</t>
+          <t>MALEKI, MEHRDAD | KOTHALE, NITISH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>本申请涉及一种用于量子计算测控的集成滤波放大装置，包括：装置壳体、电路板、前端衰减组件、前端带通滤波组件、微波放大组件、后端衰减组件和后端带通滤波组件，前端带通滤波组件、前端衰减组件、微波放大组件、后端衰减组件和后端带通滤波组件，依次连接设置在所述电路板上，且均集成在装置壳体内，通过集成带通滤波器、衰减器和微波放大器的微波前端模块，极大降低了外部线路复杂性，且该集成前端模块体积小，可直接集成到电子学设备中，使得测控脉冲从电子学设备中发生后可直接接入稀释制冷机内，极大简化了外部接线，提升了系统可靠性。</t>
+          <t>一种利用量子系统存储训练模型的方法 400 包括:接收 404 至少一个代表训练模型的参数集,该至少一个参数集包含一个或多个参数;基于该至少一个参数集生成 406 至少一个纠缠态;以及将该至少一个纠缠态存储 408 于量子系统中。通过测量该纠缠态,可以确定该至少一个参数集中的至少一个参数。</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=02fd591a-9387-4d8e-abef-42688565ec39&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=Y4mWB4Qgq0ZN0ZF5c9ezw5g6r96S%2FlAdiLwncSSBkfo%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=7042cefd-dbf9-4dc0-9986-4066c797dacb&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=hooi9d145BlHbvp5hiMpYPi36uudoDuUhSK4%2BH%2B3ZfU%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>量子自旋液体中的拓扑量子比特</t>
+          <t>作业调度程序、作业调度方法和信息处理设备</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>哈佛大学校长及研究员协会 | 麻省理工学院</t>
+          <t>富士通株式会社</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ルーキン,ミハイル,ディー. | ヴュレティック,ヴラダン | グライナー,マルクス | ベレセン,ルーベン | ビシュワナート,アシュビン | コントレラス,アレキサンダー キースリング | レビン,ハリー,ジェイ | セメギニ,ジュリア | ワン,タウト タオタオ | オムラン,アーメド | ブルブスタイン,ドレフ | エバディ,セパー</t>
+          <t>NODA, KUNIHIRO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>在一个实施例中,提供了一种装置,该装置包括二维粒子阵列,每个粒子包含: 
- [公式 1] 
- TIFF2023552091000460.tif8150;每个粒子具有第一态和激发态;属于红宝石晶格至少三个晶胞的每个粒子具有足够的阻塞半径,当处于激发态时,可以阻止红宝石晶格中至少六个最近邻粒子从其第一态跃迁到其激发态,并且该阵列具有至少一个外边缘,配置为处于第一边界条件。</t>
+          <t>量子计算任务得以高效执行。信息处理装置(10)将指示执行量子计算的任务(3a,3b)放入第一队列(1)。信息处理装置(10)将第一队列(1)中的每个任务(4a至4d)的量子计算过程转换为量子计算机(6)可执行的指令序列。信息处理装置(10)将转换完成的任务(4a至4d)放入第二队列(2)。信息处理装置(10)根据预定标准,从第二队列(2)的队首依次选择每个任务(5a至5d),确定用于执行该任务的量子比特以及是否立即执行该任务。信息处理装置(10)在确定任务需要立即执行后,指示量子计算机(6)执行该任务。</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=16e4dc1c-3013-41eb-91c4-0e2bc35596d1&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=sj1sEqHYPP7crG2lXPyE2kDFi9zchD9Go8aJv4DyFJ0%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=2c1a0b60-a7e0-46a1-af8d-2b1090e2e607&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=2MnEtmUDx8zJxGQZoQLzRsmJlcPLfXpNAYfboFFuuRM%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>转译过程中的手动量子比特映射</t>
+          <t>量子计算控制装置、量子计算机及量子计算控制方法</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>戴尔产品有限公司</t>
+          <t>独立行政法人科学技术振兴机构</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HEALY, BRENDAN BURNS | TEIXEIRA DE ABREU PINHO, RÔMULO | FONG, VICTOR</t>
+          <t>中村泰信 | 田渊丰 | 玉手修平</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -668,29 +666,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>一种方法包括:获取待映射到量子电路相应虚拟量子比特的物理量子比特的误差信息;基于这些误差信息对物理量子比特进行采样;将虚拟量子比特映射到采样得到的物理量子比特;以及对采样得到的物理量子比特执行一次量子电路。这些操作可以重复执行n次,直到获得可接受的量子电路执行结果。</t>
+          <t>量子计算控制装置具备控制信号生成部和量子比特模块。量子比特模块具备观测部、量子比特基板部、控制电路部、观测电路部以及信号处理电路部。多个量子比特分组为由各量子比特彼此的位置关系相同的多个量子比特构成的多个组而配置在量子比特基板部上。控制信号生成部生成控制信号和命令信号，控制信号用于执行一个以上的种类的空间上均匀的第一操作及以比一个以上的种类的第一操作低的频度来进行的空间上不均匀的第二操作，命令信号用于使控制电路部执行第一操作及第二操作的控制，该第一操作及第二操作是针对量子比特基板部上的量子比特的操作。控制电路部将控制信号分支到组，根据命令信号，对控制信号向量子比特基板部上的各量子比特的送出进行控制。观测电路部观测接受了第一操作或第二操作的各量子比特的状态。信号处理电路部向观测部发送各量子比特的观测信号。</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=3d214994-e647-41da-b11b-9b048d2a7d08&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=2B9SaHQRQETEbhhaTk%2FXM877NJgEZDaUpN%2FMi7BHWaQ%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=efec951d-1740-473f-842d-97180ce3a76d&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=cWStYX30VcRxj2P%2BjMY8Zcter538VTu%2BbtjG7vto470%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>结合量子计算、博弈论优化及相关方法的射频信号分类装置</t>
+          <t>原子的电子态分离器、原子干涉仪、原子跃迁频率测量装置、原子振荡器、光晶格钟、量子计算机及原子的电子态叠加态的生成方法</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>伊格尔科技有限责任公司</t>
+          <t>国立大学法人东京大学</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LAU, CHAD | RAHMES, MARK D. | CHESTER, DAVID B. | GARRETT, MICHAEL C.</t>
+          <t>香取秀俊</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -705,29 +703,29 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>一种射频(RF)信号分类装置可包括:射频接收器,用于接收射频信号;量子计算电路,用于执行量子子集求和;以及处理器。该处理器可配置为:为多个不同的深度学习模型生成博弈论奖励矩阵;与量子计算电路协作,对该博弈论奖励矩阵执行量子子集求和;基于该量子子集求和结果,从多个深度学习模型中选择一个;以及使用所选的深度学习模型处理射频信号,以进行射频信号分类。</t>
+          <t>本发明的原子的电子态分离器(1)包括：原子供给部(11)、原子移动路径(12)、探测激光光源(13)和磁场生成部(M)。原子供给部(11)供给以一定速度在原子移动路径(12)中移动的原子。探测激光光源(13)向原子移动路径(12)内供给与原子移动路径(12)同轴地在与原子的运动方向相反或相同的方向上传播的探测激光。磁场生成部(M)通过在原子移动路径(12)中生成与原子移动路径(12)正交的磁场并进行与容许电偶极子跃迁的电子态的波函数混合，能够进行基于在时间和空间上同样的探测激光的时钟跃迁的脉冲激发。或者，磁屏蔽件通过屏蔽在原子移动路径(12)中施加的磁场并在空间上改变塞曼频移，从而能够通过在时间和空间上同样的探测激光对时钟跃迁进行脉冲激发。其结果，能够连续地进行原子跃迁的分光和探测激光的频率控制，提高原子钟的稳定度。</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=494c5522-0862-40b4-9e48-8eede396c76b&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=gFV1pUFHsr%2BTO14GvyYlrExaQaex6lQray4estnB0Jc%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=826fc8c9-43e7-46de-ba8a-7944a1978dc4&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=LlykcgPkjh3vLSNIh6JaxjqICxUxQMbBk6mblb38Uwg%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>量子比特注册表命名空间</t>
+          <t>基于FPGA的蒙特卡罗路径积分-模拟量子退火方法及系统</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>红帽公司</t>
+          <t>西安电子科技大学</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GRIFFIN, LEIGH | COADY, STEPHEN</t>
+          <t>朱畅华 | 李帅威 | 何先灯 | 魏建涛 | 权东晓 | 易运晖 | 赵楠 | 陈南</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -742,12 +740,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>量子计算设备从对应于第一量子过程的第一量子指令文件(QIF)中获取第一量子过程所需的量子比特数量。该量子计算设备在包含多个量子比特注册表项的量子比特注册表中创建第一命名空间,每个注册表项对应于多个量子比特中的一个量子比特,该第一命名空间指向多个量子比特中的第一子集,该第一子集包含至少第一量子过程所需的量子比特数量。该量子计算设备将第一命名空间的标识符插入到第一QIF中。当第一QIF执行时,该量子计算设备使量子比特注册表向第一量子过程提供对第一命名空间的访问权限。</t>
+          <t>本发明公开了一种基于FPGA实现的蒙特卡罗路径积分‑模拟量子退火方法，主要解决现有蒙特卡罗路径积分‑模拟量子退火算法在CPU上运行时间效率低的问题，其实现方案包括:在Bram空间初始化原始矩阵；FPGA产生随机数以对原始矩阵进行随机操作得到新矩阵；并行计算新矩阵和原始矩阵势能项差值、动能项差值和哈密顿量差值；判断是否更新原始矩阵；选择执行更新操作后原始矩阵中势能项最小的矩阵作为当前的最优方案解；更新耦合系数不断进行迭代直到设定的迭代次数，得到最优解即为最终的最优路径。本发明大幅提升了运行的时间效率，相对于传统的蒙特卡罗路径积分‑模拟量子退火算法运行时间提高了79倍，可用于实时性要求高场景的无人机路由规划。</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=6e9dd29e-9742-4463-ad18-2eb4df554e2f&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=CmlCg9NACI2sRKU5A8xtBPEjkYDj8rCk0aTVvbWZ%2Fk4%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=4995bc0f-40ae-45ff-a154-7460d307f8a1&amp;shareId=1FE8B6DF-4B44-81FE-235C-3B3890D5E284&amp;from=EXPORT&amp;signature=mw%2F8XzKpXOlI5GwRkITNxI8qXk7gfaPvM1rU8BWWW%2BY%3D&amp;expire=94608000&amp;date=20260529T004546Z&amp;version=1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rename patent xlsx files to standardized pinyin-prefixed names
- 低温环境系统专利推送.XLSX -> patents_低温环境系统.xlsx
- 全球量子软件与算法专利情报推送.XLSX -> patents_量子软件与算法.xlsx
- 超导量子测控技术专利推送.XLSX -> patents_超导量子测控技术.xlsx
- 量子科技长三角产业创新中心公开专利.XLSX -> patents_量子科技长三角产业创新中心.xlsx
- 量子算力网专利每周推送.XLSX -> patents_量子算力网.xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/weekly_temp/patents_量子软件与算法.xlsx
+++ b/weekly_temp/patents_量子软件与算法.xlsx
@@ -493,59 +493,59 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>通过量子计算和量子通信的分布式机器学习</t>
+          <t>一种混合量子集成学习与MedMamba协同的医学图像分类方法</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>谷歌有限责任公司</t>
+          <t>重庆师范大学</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GILBOA, DAR | MCCLEAN, JARROD RYAN</t>
+          <t>董玉民 | 吴高杰</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>公开专利</t>
+          <t>授权专利</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>一个实施例包括一种方法,该方法包括在具有多个量子节点和量子通信网络的分布式量子计算系统 (DQCS) 上接收第一输入。基于第一输入和一个模型,在多个节点中的第一个量子节点上执行第一量子计算。第一量子计算的输出通过量子通信网络传输到多个量子节点中的第二个量子节点。基于第一量子计算的输出和在第二量子节点上实施的量子断层扫描算法,计算出分布式计算的结果。</t>
+          <t>本发明涉及医学图像分类技术领域，具体涉及一种混合量子集成学习与MedMamba协同的医学图像分类方法，包括将医学原始图像输入到预设的U‑Net特征提取器中，从医学原始图像中提取与特定疾病相关的可解释特征，输出对应的特征向量；将输出的特征向量输入到预先训练完成的混合量子集成学习模型中，输出对应的第一预测分类概率；将医学原始图像输入到预设的MedMamba模型，输出对应的第二预测分类概率；根据输出的第一预测分类概率和第二预测分类概率，基于预设的医学图像分类概率融合计算公式，计算出该医学原始图像所对应的最终分类概率。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=41983739-7b03-4a29-8a94-d42bd288f1c3&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=x2zwu5O68qAiOi1FfzjLIcHII840OPb%2BA%2BBRigla0v4%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=d4645b8f-948b-4f7c-94eb-d26e01cf645c&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=2IQKwh78EKfMwPKLHW8QbOFFwRyLz%2BgowZdt0cqiglI%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>光纤型激光功率量子控制装置、方法、激光发射设备</t>
+          <t>一种利用噪声诱导谱滤波效应的量子算法及系统</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>北京无线电计量测试研究所</t>
+          <t>中国科学院物理研究所</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>纪仟仟 | 薛潇博 | 韩蕾 | 申彤 | 苏亚北 | 张升康 | 葛军</t>
+          <t>张士欣</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -555,29 +555,29 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>本说明书公开了一种光纤型激光功率量子控制装置、方法、激光发射设备，以提高激光功率的抗干扰能力和稳定度。本发明装置包括：第一支路，配置为对激光器输出的激光，经过声光调制器输出0级衍射光，经光纤隔离器后输出待稳功率激光；第二支路为反馈调节支路，将第一支路中的待稳功率激光作为监测信号，导入原子钟使原子钟的输出频率随之改变，基于该输出频率与给定输出频率之间的偏差，通过反馈控制方法对第一支路中激光偏振态进行调整，以稳定输出激光的功率。本发明中，使用全光纤结构的量子控制装置具有结构简单、体积小巧、成本低、重量轻、实验装置难度低、免于调试空间光路、不易受外界杂散光影响的优势，并且提高了激光功率稳定度。</t>
+          <t>本发明提供一种利用噪声诱导谱滤波效应的量子算法，用于优化目标量子线路以获得目标量子线路的全局最优解，包括：S1、为待优化的目标量子线路构建添加量子噪声的含噪代理模型，以用于代理每一个量子逻辑门操作后量子态受噪声影响的演化过程；S2、在包含量子噪声的代理模型上进行第一次梯度下降优化处理，以获得目标量子线路的预训练线路参数；S3、将预训练线路参数加载至模拟目标量子线路的无噪或低噪环境中以完成参数迁移；S4、在完成参数迁移的模拟目标量子线路的环境中，基于目标量子线路的损失函数对第二次线路参数做梯度下降直至收敛以获得目标量子线路的全局最优解。</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=819b526b-053e-44fe-abb9-bc58efecb2c1&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=eDjSYHnwujwUnfnLRX7a6lcTR7W36aTMxSFLUA%2BMZtU%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=24cbbb68-c81d-4b5b-b94a-2be4e49de07d&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=VCjvMWx4jFgCYc3vRdRVn7FSnZLpmMAw1FN4plCYmA4%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>偏振控制的激光功率量子稳定装置、方法、激光发射设备</t>
+          <t>量子系统中用于学习双能级系统缺陷的系统和方法</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>北京无线电计量测试研究所</t>
+          <t>谷歌有限责任公司</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>纪仟仟 | 薛潇博 | 韩蕾 | 申彤 | 苏亚北 | 张升康 | 葛军</t>
+          <t>NIU, YUEZHEN | SMELYANSKIY, VADIM | BOIXO CASTRILLO, SERGIO | KLIMOV, PAUL VICTOR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -592,29 +592,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>本说明书公开了一种偏振控制的激光功率量子稳定装置、方法、激光发射设备，以提高激光功率的稳定性。本发明装置包括：激光功率调整单元，配置为对激光器输出的线偏振光，采用偏振控制器进行激光偏振态的调整，并经保偏传输后输出待稳功率激光；反馈控制单元，配置为以待稳功率激光作为监测对象，将其导入原子钟，使原子钟输出频率随之改变，基于该输出频率与给定输出频率之间的偏差，通过反馈控制方法对激光功率调整单元中激光偏振态进行调整，以稳定输出激光的功率。本发明抗环境干扰能力强、减小了传统方法里激光偏振变化对功率稳定的影响，提高了系统稳定功率微小变化的灵敏度和响应能力，更加精准的进行稳定激光功率的控制。</t>
+          <t>本公开的示例性方面提供了用于学习量子计算系统模型的机器学习模型参数的系统和方法。具体而言,本公开的示例性方面涉及用于学习深度神经网络的系统和方法,该深度神经网络配置为预测物理模型的参数值,该物理模型模拟量子门运行期间一个或多个量子比特与一个或多个双能级系统(TLS)缺陷之间相互作用的量子动力学,并通过进化算法实现。</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=676a11df-8175-4c2e-a0bf-56f414fb96a8&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=VSiYnCmNha%2BQaeQPLSGbuT%2FMEBPmMphs47whZ4h3atw%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=c6ef9718-67a1-4f38-aa10-389e62c2a090&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=tpFIzDWosEvWVa%2FVDhcYRV7kjTfqt3DHk5CkfOjOxvw%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>太赫兹光谱量子弱测量方法、系统及应用</t>
+          <t>多特征值的量子相位估计</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>中国科学院深圳先进技术研究院</t>
+          <t>谷歌有限责任公司</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>常天英 | 崔洪亮 | 路星星 | 魏东山 | 汪岳峰</t>
+          <t>BABBUSH, RYAN | DING, NAN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -629,29 +629,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>本发明提供了太赫兹光谱量子弱测量方法、系统及应用，属于太赫兹技术领域，该太赫兹光谱量子弱测量方法应用于太赫兹光谱量子弱测量系统，所述系统包括第一偏振片、第二偏振片、太赫兹时域光谱单元、发射端、探测端及样品载体，本发明提出的基于量子弱值放大效应的太赫兹量子弱测量方法及系统，能够突破目前太赫兹技术的痕量检测极限。本发明通过选定一个太赫兹偏振状态(前选态)，被测量的微小变化对其产生一种“微”扰动，再用强测量将被扰动系统态投影到后选态上，进而建立太赫兹量子弱测量体系；大多手性药物在太赫兹波段具有共振吸收性，有益于利用手性分子的旋光度微变化作为弱耦合作用，实现手性药物的高灵敏构象识别。</t>
+          <t>用于量子相位估计的方法、系统和装置。在一个方面,一种装置包括:量子电路,该量子电路包括:第一量子寄存器,该第一量子寄存器包含至少一个辅助量子比特;量子门,该量子门至少包含:(i) 两个哈达玛门,(ii) 一个相位门,(iii) 一个酉算符,以及 (iv) 一个测量算符;第二量子寄存器,该第二量子寄存器包含一个或多个量子比特,其中,该第二量子寄存器被制备在任意量子态,该任意量子态并非酉算符的本征态;以及相位学习系统,该系统配置为对所述量子电路执行相位估计实验,其包括:在每次相位估计实验中重复测量辅助量子比特的状态,以确定辅助量子比特状态的期望值并学习酉算符本征值的相位。</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=c9746448-bedc-4316-b621-fe01a87980db&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=wi1MMHbFVv7qi%2BmluFU5HXTRO59DnQ5Cn1nbNzzY1ak%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=3ff4d9b9-bee4-4f43-a63e-83697c266b42&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=mp3sCPeem1ukTRJoe96BsI2l6e%2FQinIqLtMHn%2BRHjDw%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>蛋白质DDG预测模型优化方法、蛋白质DDG预测方法及相关装置</t>
+          <t>处理表面代码匹配图中高亮顶点的垂直对</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>上海图灵智算量子科技有限公司 | 图灵智算量子科技(无锡)有限公司</t>
+          <t>亚马逊科技公司</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>丁灏 | 陆遥遥 | 唐可馨</t>
+          <t>CHAMBERLAND, CHRISTOPHER | GONCALVES, LUIS | SIVARAJAH, PRASAHNT | PETERSON, ERIC CHRISTOPHER | GRIMBERG, SEBASTIAN JOHANNES</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -666,29 +666,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>本发明的实施例提供了一种蛋白质DDG预测模型优化方法、蛋白质DDG预测方法及相关装置，涉及生物信息数据处理技术领域。该方法包括：获取野生型蛋白质三维结构数据、突变体蛋白质三维结构数据以及第一DDG值。分别将野生型蛋白质三维结构数据与突变体蛋白质三维结构数据输入蛋白质DDG初始预测模型中优化后的编码器，得到野生型蛋白质三维结构数据对应的第一特征向量以及突变体蛋白质三维结构数据对应的第二特征向量。基于变分量子线路，根据第一特征向量以及第二特征向量得到第二DDG值。根据第一DDG值与第二DDG值对蛋白质DDG初始预测模型进行迭代优化，得到蛋白质DDG预测模型。本发明可以有效提高蛋白质DDG的预测准确率。</t>
+          <t>本发明公开了用于降低量子表面码电路级噪声量子纠错过程中,经过第一解码阶段(例如,通过本地解码器)后,多轮伴随式测量结果的伴随式密度的技术。这些降低伴随式密度的技术可以包括伴随式坍缩和/或垂直清理技术。在伴随式坍缩技术中,可以将测量结果体分割成多个片层,然后对各个片层进行坍缩,从而移除垂直方向上的突出显示顶点对。在垂直清理技术中,可以在第一解码阶段之后,直接从匹配图中移除垂直方向上的突出显示顶点对。移除垂直方向上的突出显示顶点对之后,测量结果将在第二全局解码阶段进行解码。这种技术能够实现快速解码,并降低使用量子表面码实现的量子算法的纠错轮次延迟时间。</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=672fd6cf-6f0e-41fc-8e84-33a2e4bdaf83&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=d02VwQytTfhj8BUFbVzJ6%2BlEuDDqhl88coYfbn6GIkc%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=96463724-9d1a-4d5a-aa6c-f0cb66a03c97&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=GiTw1TTaYYBdtJUzMrqsSFBxcCJdNcz%2B7jZXuZxHhqo%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>一种混合量子集成学习与MedMamba协同的医学图像分类方法</t>
+          <t>一种用于求解离散二次模型的混合算法的系统和方法</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>重庆师范大学</t>
+          <t>D WAVE 系统公司</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>董玉民 | 吴高杰</t>
+          <t>エスファハニ,ホセイン,サデギ | ベルヌーディ,ウィリアム,ダヴリュー. | ラーマニ,モーセン</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -698,34 +698,35 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>本发明涉及医学图像分类技术领域，具体涉及一种混合量子集成学习与MedMamba协同的医学图像分类方法，包括将医学原始图像输入到预设的U‑Net特征提取器中，从医学原始图像中提取与特定疾病相关的可解释特征，输出对应的特征向量；将输出的特征向量输入到预先训练完成的混合量子集成学习模型中，输出对应的第一预测分类概率；将医学原始图像输入到预设的MedMamba模型，输出对应的第二预测分类概率；根据输出的第一预测分类概率和第二预测分类概率，基于预设的医学图像分类概率融合计算公式，计算出该医学原始图像所对应的最终分类概率。</t>
+          <t>采用吉布斯采样和交叉玻尔兹曼更新法求解离散二次模型。 
+该方法基于每个变量与其他变量的相互作用,计算每个变量各状态的能量,计算指数权重,并计算与该指数权重成正比的归一化概率。每个变量的能量是根据其自身大小和所有其他变量的当前状态计算的,计算指数权重,计算每个变量的可行域,并计算与该指数权重和所满足的约束条件成正比的归一化概率。该方法通过混合计算系统执行,为每个变量获得两个候选值,构建一个使用二进制值来确定每个变量应取哪个候选值的哈密顿量,然后基于该哈密顿量构建一个二维二次模型。通过量子处理器从该二维二次模型中获取样本。</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=d4645b8f-948b-4f7c-94eb-d26e01cf645c&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=2IQKwh78EKfMwPKLHW8QbOFFwRyLz%2BgowZdt0cqiglI%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=b5843080-6f14-46bd-a875-ecfa9ca57327&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=vV8i09e1sZvHnlordWP6TkjMzkk%2FxFyzW0zW%2FSPCnWM%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>面向mRNA编码蛋白结构预测的智能算力调度系统和方法</t>
+          <t>磁化自旋量子人工神经网络装置</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>微观纪元(合肥)量子科技有限公司</t>
+          <t>EFRAM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>郑跃强 | 夏坚 | 管佳明 | 董景祥</t>
+          <t>강희복</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -735,17 +736,23 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>本发明公开了一种面向mRNA编码蛋白结构预测的智能算力调度系统、方法和电子设备，面向mRNA编码蛋白结构预测的智能算力调度系统包括：输入与任务管理层，用于获取并翻译mRNA序列，得到原子性子任务；智能感知与调度核心层，与输入与任务管理层连接，用于根据原子性子任务，生成对应的优化调度决策；异构算力资源层，与智能感知与调度核心层，用于根据优化调度决策，进行经典计算和/或量子计算，得到对应的经典计算结果和/或量子计算结果；输出与优化层，与异构算力资源层连接，用于根据经典计算结果和/或量子计算结果，生成蛋白质3D结构模型。本发明的系统能够提高蛋白结构预测结果的准确性、效率，还能够提高算力资源利用率。</t>
+          <t>一个线性组合(48)节点、一个激活函数(49)、一个输出数据(Y1)、m 个输入数据 Xi 终端和 m 个权重区域(400)元素构成一个独立的层。 
+换句话说,该装置是通过形成与输出数据数量 (Yi) 相等的独立层来构建的。 
+例如,如果由 n 个输出数据 (Yn) 组成,则该设备由形成 n 个独立层构成。 
+当由 m 个输入数据 Xi 端子和 n 个输出数据 (Yn) 端子组成时,该设备通过形成 n 个独立层进行配置。 
+ m 个输入数据端子 Xi 通过 TLV(层直通)连接到 n 个独立的层。 
+例如,第一个输入端子 X1 通过 TLV(层通孔)连接到 n 个独立的层。 
+此外,第 m 个输入值 Xm 端子的特点是,它通过 TLV(层间过孔)与 n 个独立的层中的每一个都相连。</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=4d22a8d3-adf5-47dc-9aed-5c7d59d46b35&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=axXXCq5IhvK07YTz55KsVaL1hHumCPG6xLS3XnMhQoc%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=0b17bd05-b7e9-471d-830e-01cd79f8a5c6&amp;shareId=1B475C3G-7GDG-8976-149D-791913G50906&amp;from=EXPORT&amp;signature=4ZmPz4kCFhX3NXF%2Fsvdo8zYjUmJ7GW%2BWZQsGLW7qNos%3D&amp;expire=94608000&amp;date=20260605T004519Z&amp;version=1.0</t>
         </is>
       </c>
     </row>

</xml_diff>